<commit_message>
update on making contin ndwi data
made a couple of updated files on ndwi for making continuous ndwi value regressions/ correlations on nematodes
</commit_message>
<xml_diff>
--- a/Metadata/Metadata spreadsheet w NDWI 20203.xlsx
+++ b/Metadata/Metadata spreadsheet w NDWI 20203.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29325"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8F9CAB0D-7866-4840-AFDB-FD5BEF85761B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{86F019DC-3CBD-49EC-B36E-951C1A0385D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="35">
   <si>
     <t>Farms</t>
   </si>
@@ -48,7 +48,7 @@
     <t>Longitude</t>
   </si>
   <si>
-    <t>NDWI</t>
+    <t>NDWI avg</t>
   </si>
   <si>
     <t>NDWI 1</t>
@@ -58,6 +58,12 @@
   </si>
   <si>
     <t>NDWI 3</t>
+  </si>
+  <si>
+    <t>rootknot</t>
+  </si>
+  <si>
+    <t>spiral</t>
   </si>
   <si>
     <t>Turf Farm</t>
@@ -174,11 +180,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -514,13 +521,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="17.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:11">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -548,16 +555,22 @@
       <c r="I1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:9">
+      <c r="J1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B2">
         <v>2023</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D2" s="1">
         <v>31.237396</v>
@@ -578,16 +591,22 @@
       <c r="I2" s="2">
         <v>0.52582387165490596</v>
       </c>
-    </row>
-    <row r="3" spans="1:9">
+      <c r="J2" s="3">
+        <v>241</v>
+      </c>
+      <c r="K2" s="3">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B3">
         <v>2023</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D3" s="1">
         <v>31.457160999999999</v>
@@ -608,16 +627,22 @@
       <c r="I3" s="2">
         <v>0.104537834466986</v>
       </c>
-    </row>
-    <row r="4" spans="1:9">
+      <c r="J3" s="3">
+        <v>16</v>
+      </c>
+      <c r="K3" s="3">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B4">
         <v>2023</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D4" s="1">
         <v>31.170497999999998</v>
@@ -638,16 +663,22 @@
       <c r="I4" s="2">
         <v>0.544776410416143</v>
       </c>
-    </row>
-    <row r="5" spans="1:9">
+      <c r="J4" s="3">
+        <v>253</v>
+      </c>
+      <c r="K4" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
       <c r="A5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5">
+        <v>2023</v>
+      </c>
+      <c r="C5" t="s">
         <v>14</v>
-      </c>
-      <c r="B5">
-        <v>2023</v>
-      </c>
-      <c r="C5" t="s">
-        <v>12</v>
       </c>
       <c r="D5" s="1">
         <v>31.427333000000001</v>
@@ -668,16 +699,22 @@
       <c r="I5" s="2">
         <v>0.448046205974099</v>
       </c>
-    </row>
-    <row r="6" spans="1:9">
+      <c r="J5" s="3">
+        <v>119</v>
+      </c>
+      <c r="K5" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B6">
         <v>2023</v>
       </c>
       <c r="C6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D6" s="1">
         <v>31.389348999999999</v>
@@ -698,16 +735,22 @@
       <c r="I6" s="2">
         <v>0.422369192866346</v>
       </c>
-    </row>
-    <row r="7" spans="1:9">
+      <c r="J6" s="3">
+        <v>250</v>
+      </c>
+      <c r="K6" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B7">
         <v>2023</v>
       </c>
       <c r="C7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D7" s="1">
         <v>31.235600999999999</v>
@@ -728,16 +771,22 @@
       <c r="I7" s="2">
         <v>0.42661671857091699</v>
       </c>
-    </row>
-    <row r="8" spans="1:9">
+      <c r="J7" s="3">
+        <v>235</v>
+      </c>
+      <c r="K7" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B8">
         <v>2023</v>
       </c>
       <c r="C8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D8" s="1">
         <v>31.448412999999999</v>
@@ -758,16 +807,22 @@
       <c r="I8" s="2">
         <v>0.48585809216081399</v>
       </c>
-    </row>
-    <row r="9" spans="1:9">
+      <c r="J8" s="3">
+        <v>118</v>
+      </c>
+      <c r="K8" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B9">
         <v>2023</v>
       </c>
       <c r="C9" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D9" s="1">
         <v>31.428485999999999</v>
@@ -788,16 +843,22 @@
       <c r="I9" s="2">
         <v>0.37796841854250501</v>
       </c>
-    </row>
-    <row r="10" spans="1:9">
+      <c r="J9" s="3">
+        <v>0</v>
+      </c>
+      <c r="K9" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B10">
         <v>2023</v>
       </c>
       <c r="C10" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D10" s="1">
         <v>31.175878999999998</v>
@@ -818,16 +879,22 @@
       <c r="I10" s="2">
         <v>0.42471898408692499</v>
       </c>
-    </row>
-    <row r="11" spans="1:9">
+      <c r="J10" s="3">
+        <v>0</v>
+      </c>
+      <c r="K10" s="3">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
       <c r="A11" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B11">
         <v>2023</v>
       </c>
       <c r="C11" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D11" s="1">
         <v>31.319068000000001</v>
@@ -848,16 +915,22 @@
       <c r="I11" s="2">
         <v>0.37638796963103099</v>
       </c>
-    </row>
-    <row r="12" spans="1:9">
+      <c r="J11" s="3">
+        <v>247</v>
+      </c>
+      <c r="K11" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B12">
         <v>2023</v>
       </c>
       <c r="C12" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D12" s="1">
         <v>31.301092000000001</v>
@@ -878,16 +951,22 @@
       <c r="I12" s="2">
         <v>0.52463916569459101</v>
       </c>
-    </row>
-    <row r="13" spans="1:9">
+      <c r="J12" s="3">
+        <v>74</v>
+      </c>
+      <c r="K12" s="3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
       <c r="A13" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B13">
         <v>2023</v>
       </c>
       <c r="C13" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D13" s="1">
         <v>31.237894000000001</v>
@@ -908,16 +987,22 @@
       <c r="I13" s="2">
         <v>0.48806970462568799</v>
       </c>
-    </row>
-    <row r="14" spans="1:9">
+      <c r="J13" s="3">
+        <v>254</v>
+      </c>
+      <c r="K13" s="3">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11">
       <c r="A14" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B14">
         <v>2023</v>
       </c>
       <c r="C14" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D14" s="1">
         <v>31.239789999999999</v>
@@ -938,16 +1023,22 @@
       <c r="I14" s="2">
         <v>0.32451446917990201</v>
       </c>
-    </row>
-    <row r="15" spans="1:9">
+      <c r="J14" s="3">
+        <v>4</v>
+      </c>
+      <c r="K14" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11">
       <c r="A15" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B15">
         <v>2023</v>
       </c>
       <c r="C15" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D15" s="1">
         <v>31.448384000000001</v>
@@ -968,16 +1059,22 @@
       <c r="I15" s="2">
         <v>0.43225743086702001</v>
       </c>
-    </row>
-    <row r="16" spans="1:9">
+      <c r="J15" s="3">
+        <v>0</v>
+      </c>
+      <c r="K15" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11">
       <c r="A16" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B16">
         <v>2023</v>
       </c>
       <c r="C16" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D16" s="1">
         <v>31.224142000000001</v>
@@ -998,16 +1095,22 @@
       <c r="I16" s="2">
         <v>0.443355651973868</v>
       </c>
-    </row>
-    <row r="17" spans="1:9">
+      <c r="J16" s="3">
+        <v>0</v>
+      </c>
+      <c r="K16" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11">
       <c r="A17" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B17">
         <v>2023</v>
       </c>
       <c r="C17" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D17" s="1">
         <v>31.316875</v>
@@ -1028,16 +1131,22 @@
       <c r="I17" s="2">
         <v>0.28529136312624698</v>
       </c>
-    </row>
-    <row r="18" spans="1:9">
+      <c r="J17" s="3">
+        <v>67</v>
+      </c>
+      <c r="K17" s="3">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11">
       <c r="A18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B18">
         <v>2023</v>
       </c>
       <c r="C18" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D18" s="1">
         <v>31.411767999999999</v>
@@ -1058,16 +1167,22 @@
       <c r="I18" s="2">
         <v>0.47919128174182801</v>
       </c>
-    </row>
-    <row r="19" spans="1:9">
+      <c r="J18" s="3">
+        <v>231</v>
+      </c>
+      <c r="K18" s="3">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11">
       <c r="A19" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B19">
         <v>2023</v>
       </c>
       <c r="C19" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D19" s="1">
         <v>31.231984000000001</v>
@@ -1088,16 +1203,22 @@
       <c r="I19" s="2">
         <v>0.47646586620895098</v>
       </c>
-    </row>
-    <row r="20" spans="1:9">
+      <c r="J19" s="3">
+        <v>2</v>
+      </c>
+      <c r="K19" s="3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11">
       <c r="A20" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B20">
         <v>2023</v>
       </c>
       <c r="C20" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D20" s="1">
         <v>31.204640000000001</v>
@@ -1118,16 +1239,22 @@
       <c r="I20" s="2">
         <v>0.48320652039133499</v>
       </c>
-    </row>
-    <row r="21" spans="1:9">
+      <c r="J20" s="3">
+        <v>4</v>
+      </c>
+      <c r="K20" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11">
       <c r="A21" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B21">
         <v>2023</v>
       </c>
       <c r="C21" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D21" s="1">
         <v>31.423584999999999</v>
@@ -1147,6 +1274,12 @@
       </c>
       <c r="I21" s="2">
         <v>0.33956178972275802</v>
+      </c>
+      <c r="J21" s="3">
+        <v>0</v>
+      </c>
+      <c r="K21" s="3">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>